<commit_message>
Bỏ tên đích danh sản phẩm đối thủ khỏi tài liệu định hướng
Thay "Simply Piano và tương tự" bằng mô tả theo cách làm là "app học
đàn tự động chấm điểm". Lập luận không yếu đi vì người đọc từng dùng
loại app này sẽ tự nhận ra.

Ghi lại quy tắc không nêu tên thương hiệu đối thủ ở mọi nơi kèm cơ sở
pháp lý: Luật Quảng cáo sửa đổi 2025 chỉ còn cấm so sánh không có tài
liệu chứng minh, nhưng trải nghiệm cá nhân không phải tài liệu chứng
minh nên vẫn vướng; Nghị định 38/2021 phạt 40-60 triệu với cá nhân;
Luật Cạnh tranh 2018 Điều 45 cấm so sánh không có bằng chứng.

Thêm quy tắc này vào AGENTS.md để không bị gắn tên lại về sau.
</commit_message>
<xml_diff>
--- a/docs/_internal/uoc-tinh-doanh-thu.xlsx
+++ b/docs/_internal/uoc-tinh-doanh-thu.xlsx
@@ -9,7 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Mô hình" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Ghi chú" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Đòn bẩy" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Thuê bao" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Ghi chú" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
   <si>
     <t xml:space="preserve">Ước tính doanh thu hàng tháng — Gói Nền tảng 399.000đ</t>
   </si>
@@ -165,6 +167,231 @@
   </si>
   <si>
     <t xml:space="preserve">Ô vàng chữ xanh = bạn sửa. Ô xám/xanh lá = công thức tự tính, đừng gõ đè.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">So sánh đòn bẩy — thay đổi nào làm lợi nhuận tăng nhiều nhất?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mỗi dòng là một phương án. Chỉ những ô vàng thay đổi so với dòng 'Cơ sở'. Phí, hoàn tiền, thuế lấy từ sheet Mô hình.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phương án</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lượt truy cập</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% tạo TK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% hết Ch.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% mua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giá bán</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doanh thu thêm / khách</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chi phí cố định</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số đơn/tháng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doanh thu thuần</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CÒN LẠI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">So với Cơ sở</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cơ sở — giữ nguyên mọi thứ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A. Tăng giá lên 599k, chuyển đổi giữ nguyên</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B. Tăng giá lên 599k, chuyển đổi giảm 25%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. Sản phẩm giữ chân tốt hơn: hết Ch.1 25%→40%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D. Bán thêm Giai đoạn 3 (599k) cho 30% khách cũ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E. Gói kèm nhận xét 1-1 (10% khách mua thêm 1tr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F. Cắt hết quảng cáo, lưu lượng giảm 30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G. Tăng gấp đôi lưu lượng bằng quảng cáo 3tr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H. Kết hợp A + C + D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đọc bảng này thế nào</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Cột 'CÒN LẠI' đã trừ phí cổng, hoàn tiền, chi phí cố định và thuế 7%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 'Doanh thu thêm / khách' là tiền trung bình mỗi khách chi thêm ngoài gói Nền tảng, tính bình quân trên TOÀN BỘ khách (kể cả người không mua thêm).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Phương án B mô phỏng việc tăng giá làm mất khách: giá +50% nhưng tỷ lệ mua tụt từ 22% xuống 16,5%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Phương án E cộng thêm 200k chi phí cố định vì nhận xét 1-1 tốn thời gian thật của bạn — con số này nên tăng nếu bạn quy giờ ra tiền.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Phương án G cho thấy quảng cáo chỉ có lãi khi chi phí mỗi lượt truy cập thấp hơn dòng 'mỗi lượt truy cập đáng giá bao nhiêu' ở sheet Mô hình.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua đứt hay Thuê bao năm (kèm sheet nhạc định kỳ)?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thuê bao chỉ hợp lý khi nội dung sinh thêm liên tục. Sheet nhạc định kỳ đúng là loại đó — nên phép so sánh này mới có nghĩa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GIẢ ĐỊNH CHUNG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giá trị</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số người chạm paywall mỗi tháng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lấy từ sheet Mô hình, cột Cơ sở.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ mua — bán đứt 399k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cột Cơ sở ở sheet Mô hình.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ mua — thuê bao năm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUAN TRỌNG: người ta ngại cam kết định kỳ hơn. Đặt thấp hơn dòng trên.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giá bán đứt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giá gói năm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~50k/tháng. Cao hơn nữa thì phải so với app quốc tế.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ gia hạn sau mỗi năm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIẾN QUYẾT ĐỊNH. Sản phẩm học tập thường 20-40%. Chưa có số thật thì đừng đặt cao.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chi phí sản xuất sheet nhạc mỗi tháng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thời gian soạn + biên tập + phí bản quyền. Đây là nghĩa vụ VĨNH VIỄN.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chi phí cố định khác / tháng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hạ tầng + quảng cáo, lấy từ cột Cơ sở.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SO SÁNH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua đứt 399k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thuê bao năm 599k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khách mới mỗi tháng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doanh thu thuần / tháng — NĂM ĐẦU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Năm đầu chưa có ai gia hạn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doanh thu thuần / tháng — TRẠNG THÁI ỔN ĐỊNH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phải mất khoảng 3-4 năm mới tới được mức này.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số người đang trả tiền (ổn định)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua đứt không có khái niệm này.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giá trị vòng đời mỗi khách (LTV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chi phí cố định / tháng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thuê bao gánh thêm chi phí sản xuất sheet mãi mãi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CÒN LẠI / THÁNG — năm đầu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CÒN LẠI / THÁNG — ổn định</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ gia hạn TỐI THIỂU để thuê bao thắng mua đứt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đây là mức gia hạn tối thiểu để thuê bao đem lại lợi nhuận BẰNG mua đứt, sau khi đã trừ chi phí sản xuất sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doanh thu ổn định cần có để bù chi phí sản xuất sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nếu doanh thu tăng thêm nhờ thuê bao không vượt con số này thì bạn đang làm không công.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ĐỘ NHẠY — 'Còn lại/tháng ở trạng thái ổn định' của gói thuê bao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ gia hạn ↓ / Tỷ lệ mua thuê bao →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Điều kiện để thuê bao là quyết định đúng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Bạn phải thật sự ra sheet mới ĐỀU ĐẶN, mãi mãi. Khách trả tiền cho dòng chảy, không phải cho kho. Tháng nào không ra bài là tháng đó mất uy tín.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Bản quyền. Phối và bán sheet của ca khúc còn bảo hộ mà chưa xin phép là xâm phạm quyền tác giả — ở Việt Nam liên hệ VCPMC. An toàn tuyệt đối: dân ca, nhạc hết thời hạn bảo hộ, và sáng tác của chính bạn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Trả trước cả năm là một khoản NỢ, không phải doanh thu đã kiếm được. Bạn đang bán trước 12 tháng lao động của mình.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Bảng độ nhạy cho thấy: khi tỷ lệ mua tụt xuống 8-10% thì dù gia hạn có tốt tới đâu cũng không cứu được. Số người trả tiền quan trọng hơn tỷ lệ gia hạn.</t>
   </si>
   <si>
     <t xml:space="preserve">Đọc cái này trước khi tin bất kỳ con số nào</t>
@@ -228,15 +455,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="#,##0&quot; đ&quot;"/>
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
     <numFmt numFmtId="169" formatCode="0%"/>
+    <numFmt numFmtId="170" formatCode="\+0%;\-0%;0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -339,6 +567,12 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Cambria"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -421,7 +655,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="53">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -446,7 +680,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -551,6 +785,74 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1529,6 +1831,1058 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:L21"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="32" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="33" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="33" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="33" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" s="33" t="s">
+        <v>56</v>
+      </c>
+      <c r="H4" s="33" t="s">
+        <v>57</v>
+      </c>
+      <c r="I4" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="J4" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="K4" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="L4" s="33" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C5" s="35" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="D5" s="35" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E5" s="35" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F5" s="21" t="n">
+        <v>399000</v>
+      </c>
+      <c r="G5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="21" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="I5" s="36" t="n">
+        <f aca="false">B5*C5*D5*E5</f>
+        <v>11.55</v>
+      </c>
+      <c r="J5" s="37" t="n">
+        <f aca="false">I5*(F5+G5)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4268576.8125</v>
+      </c>
+      <c r="K5" s="17" t="n">
+        <f aca="false">J5-H5-J5*'Mô hình'!$C$26</f>
+        <v>2419776.435625</v>
+      </c>
+      <c r="L5" s="38" t="n">
+        <f aca="false">IF($K$5=0,"",K5/$K$5-1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C6" s="40" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="D6" s="40" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E6" s="40" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>599000</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="I6" s="41" t="n">
+        <f aca="false">B6*C6*D6*E6</f>
+        <v>11.55</v>
+      </c>
+      <c r="J6" s="42" t="n">
+        <f aca="false">I6*(F6+G6)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>6408214.3125</v>
+      </c>
+      <c r="K6" s="20" t="n">
+        <f aca="false">J6-H6-J6*'Mô hình'!$C$26</f>
+        <v>4409639.310625</v>
+      </c>
+      <c r="L6" s="43" t="n">
+        <f aca="false">IF($K$5=0,"",K6/$K$5-1)</f>
+        <v>0.822333355141564</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="39" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="D7" s="40" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>599000</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="I7" s="41" t="n">
+        <f aca="false">B7*C7*D7*E7</f>
+        <v>8.6625</v>
+      </c>
+      <c r="J7" s="42" t="n">
+        <f aca="false">I7*(F7+G7)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4806160.734375</v>
+      </c>
+      <c r="K7" s="20" t="n">
+        <f aca="false">J7-H7-J7*'Mô hình'!$C$26</f>
+        <v>2919729.48296875</v>
+      </c>
+      <c r="L7" s="43" t="n">
+        <f aca="false">IF($K$5=0,"",K7/$K$5-1)</f>
+        <v>0.206611255479318</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="39" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C8" s="40" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="D8" s="40" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E8" s="40" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>399000</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="I8" s="41" t="n">
+        <f aca="false">B8*C8*D8*E8</f>
+        <v>18.48</v>
+      </c>
+      <c r="J8" s="42" t="n">
+        <f aca="false">I8*(F8+G8)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>6829722.9</v>
+      </c>
+      <c r="K8" s="20" t="n">
+        <f aca="false">J8-H8-J8*'Mô hình'!$C$26</f>
+        <v>4801642.297</v>
+      </c>
+      <c r="L8" s="43" t="n">
+        <f aca="false">IF($K$5=0,"",K8/$K$5-1)</f>
+        <v>0.984333026104451</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="D9" s="40" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E9" s="40" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>399000</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>180000</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="I9" s="41" t="n">
+        <f aca="false">B9*C9*D9*E9</f>
+        <v>11.55</v>
+      </c>
+      <c r="J9" s="42" t="n">
+        <f aca="false">I9*(F9+G9)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>6194250.5625</v>
+      </c>
+      <c r="K9" s="20" t="n">
+        <f aca="false">J9-H9-J9*'Mô hình'!$C$26</f>
+        <v>4210653.023125</v>
+      </c>
+      <c r="L9" s="43" t="n">
+        <f aca="false">IF($K$5=0,"",K9/$K$5-1)</f>
+        <v>0.740100019627408</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C10" s="40" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="D10" s="40" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E10" s="40" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>399000</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>100000</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>1750000</v>
+      </c>
+      <c r="I10" s="41" t="n">
+        <f aca="false">B10*C10*D10*E10</f>
+        <v>11.55</v>
+      </c>
+      <c r="J10" s="42" t="n">
+        <f aca="false">I10*(F10+G10)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>5338395.5625</v>
+      </c>
+      <c r="K10" s="20" t="n">
+        <f aca="false">J10-H10-J10*'Mô hình'!$C$26</f>
+        <v>3214707.873125</v>
+      </c>
+      <c r="L10" s="43" t="n">
+        <f aca="false">IF($K$5=0,"",K10/$K$5-1)</f>
+        <v>0.328514413892405</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="39" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>2100</v>
+      </c>
+      <c r="C11" s="40" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="D11" s="40" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E11" s="40" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F11" s="15" t="n">
+        <v>399000</v>
+      </c>
+      <c r="G11" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="15" t="n">
+        <v>550000</v>
+      </c>
+      <c r="I11" s="41" t="n">
+        <f aca="false">B11*C11*D11*E11</f>
+        <v>8.085</v>
+      </c>
+      <c r="J11" s="42" t="n">
+        <f aca="false">I11*(F11+G11)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>2988003.76875</v>
+      </c>
+      <c r="K11" s="20" t="n">
+        <f aca="false">J11-H11-J11*'Mô hình'!$C$26</f>
+        <v>2228843.5049375</v>
+      </c>
+      <c r="L11" s="43" t="n">
+        <f aca="false">IF($K$5=0,"",K11/$K$5-1)</f>
+        <v>-0.0789051946603426</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="39" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C12" s="40" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="D12" s="40" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E12" s="40" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>399000</v>
+      </c>
+      <c r="G12" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="15" t="n">
+        <v>3550000</v>
+      </c>
+      <c r="I12" s="41" t="n">
+        <f aca="false">B12*C12*D12*E12</f>
+        <v>23.1</v>
+      </c>
+      <c r="J12" s="42" t="n">
+        <f aca="false">I12*(F12+G12)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>8537153.625</v>
+      </c>
+      <c r="K12" s="20" t="n">
+        <f aca="false">J12-H12-J12*'Mô hình'!$C$26</f>
+        <v>4389552.87125</v>
+      </c>
+      <c r="L12" s="43" t="n">
+        <f aca="false">IF($K$5=0,"",K12/$K$5-1)</f>
+        <v>0.814032406723652</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="39" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C13" s="40" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="D13" s="40" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E13" s="40" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F13" s="15" t="n">
+        <v>599000</v>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>270000</v>
+      </c>
+      <c r="H13" s="15" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="I13" s="41" t="n">
+        <f aca="false">B13*C13*D13*E13</f>
+        <v>18.48</v>
+      </c>
+      <c r="J13" s="42" t="n">
+        <f aca="false">I13*(F13+G13)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>14874759.9</v>
+      </c>
+      <c r="K13" s="20" t="n">
+        <f aca="false">J13-H13-J13*'Mô hình'!$C$26</f>
+        <v>12283526.707</v>
+      </c>
+      <c r="L13" s="43" t="n">
+        <f aca="false">IF($K$5=0,"",K13/$K$5-1)</f>
+        <v>4.07630644143673</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="26" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="1" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="32" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="18"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="44" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="8" t="n">
+        <f aca="false">'Mô hình'!C9</f>
+        <v>52.5</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="44" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="40" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="44" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="40" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="44" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>399000</v>
+      </c>
+      <c r="D8" s="9"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="44" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>599000</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="44" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" s="40" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="44" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="44" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="45" t="s">
+        <v>99</v>
+      </c>
+      <c r="B15" s="36" t="n">
+        <f aca="false">$B$5*$B$6</f>
+        <v>11.55</v>
+      </c>
+      <c r="C15" s="36" t="n">
+        <f aca="false">$B$5*$B$7</f>
+        <v>7.875</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="45" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16" s="37" t="n">
+        <f aca="false">B15*$B$8*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4268576.8125</v>
+      </c>
+      <c r="C16" s="37" t="n">
+        <f aca="false">C15*$B$9*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4369237.03125</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="26" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="20" t="n">
+        <f aca="false">B15*$B$8*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4268576.8125</v>
+      </c>
+      <c r="C17" s="20" t="n">
+        <f aca="false">C15*$B$9/(1-$B$10)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>6721903.125</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="45" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>105</v>
+      </c>
+      <c r="C18" s="47" t="n">
+        <f aca="false">C15*12/(1-$B$10)</f>
+        <v>145.384615384615</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="45" t="s">
+        <v>107</v>
+      </c>
+      <c r="B19" s="37" t="n">
+        <f aca="false">$B$8</f>
+        <v>399000</v>
+      </c>
+      <c r="C19" s="37" t="n">
+        <f aca="false">$B$9/(1-$B$10)</f>
+        <v>921538.461538462</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="45" t="s">
+        <v>108</v>
+      </c>
+      <c r="B20" s="37" t="n">
+        <f aca="false">$B$12</f>
+        <v>1550000</v>
+      </c>
+      <c r="C20" s="37" t="n">
+        <f aca="false">$B$11+$B$12</f>
+        <v>3550000</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="26" t="s">
+        <v>110</v>
+      </c>
+      <c r="B21" s="20" t="n">
+        <f aca="false">B16-B20-B16*'Mô hình'!$C$26</f>
+        <v>2419776.435625</v>
+      </c>
+      <c r="C21" s="20" t="n">
+        <f aca="false">C16-C20-C16*'Mô hình'!$C$26</f>
+        <v>513390.439062501</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="B22" s="20" t="n">
+        <f aca="false">B17-B20-B17*'Mô hình'!$C$26</f>
+        <v>2419776.435625</v>
+      </c>
+      <c r="C22" s="20" t="n">
+        <f aca="false">C17-C20-C17*'Mô hình'!$C$26</f>
+        <v>2701369.90625</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="48" t="n">
+        <f aca="false">IF(C15=0,"",1-(C15*$B$9*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)*(1-'Mô hình'!$C$26))/(B15*$B$8*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)*(1-'Mô hình'!$C$26)+$B$11))</f>
+        <v>0.319339596234463</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="45" t="s">
+        <v>114</v>
+      </c>
+      <c r="B25" s="37" t="n">
+        <f aca="false">$B$11/(1-'Mô hình'!$C$26)</f>
+        <v>2150537.6344086</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="26" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="28" t="s">
+        <v>117</v>
+      </c>
+      <c r="B28" s="29" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C28" s="29" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D28" s="29" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E28" s="29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F28" s="29" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G28" s="29" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="49" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="B29" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-1000421.68529412</v>
+      </c>
+      <c r="C29" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-363027.106617647</v>
+      </c>
+      <c r="D29" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>274367.472058824</v>
+      </c>
+      <c r="E29" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1230459.34007353</v>
+      </c>
+      <c r="F29" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2186551.20808824</v>
+      </c>
+      <c r="G29" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3461340.36544118</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="49" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B30" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-841073.040625</v>
+      </c>
+      <c r="C30" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-163841.30078125</v>
+      </c>
+      <c r="D30" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>513390.4390625</v>
+      </c>
+      <c r="E30" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1529238.04882813</v>
+      </c>
+      <c r="F30" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2545085.65859375</v>
+      </c>
+      <c r="G30" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3899549.13828125</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="49" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B31" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-660477.91</v>
+      </c>
+      <c r="C31" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>61902.6125000003</v>
+      </c>
+      <c r="D31" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>784283.135000001</v>
+      </c>
+      <c r="E31" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1867853.91875</v>
+      </c>
+      <c r="F31" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2951424.7025</v>
+      </c>
+      <c r="G31" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>4396185.7475</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="49" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B32" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-454083.474999999</v>
+      </c>
+      <c r="C32" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>319895.65625</v>
+      </c>
+      <c r="D32" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1093874.7875</v>
+      </c>
+      <c r="E32" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2254843.484375</v>
+      </c>
+      <c r="F32" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3415812.18125</v>
+      </c>
+      <c r="G32" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>4963770.44375</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="49" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B33" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-215936.05</v>
+      </c>
+      <c r="C33" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>617579.937500001</v>
+      </c>
+      <c r="D33" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1451095.925</v>
+      </c>
+      <c r="E33" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2701369.90625</v>
+      </c>
+      <c r="F33" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3951643.8875</v>
+      </c>
+      <c r="G33" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>5618675.8625</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="49" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B34" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>61902.6125000007</v>
+      </c>
+      <c r="C34" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>964878.265625001</v>
+      </c>
+      <c r="D34" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1867853.91875</v>
+      </c>
+      <c r="E34" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3222317.3984375</v>
+      </c>
+      <c r="F34" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>4576780.878125</v>
+      </c>
+      <c r="G34" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>6382732.184375</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="49" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B35" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>784283.135000001</v>
+      </c>
+      <c r="C35" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1867853.91875</v>
+      </c>
+      <c r="D35" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2951424.7025</v>
+      </c>
+      <c r="E35" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>4576780.878125</v>
+      </c>
+      <c r="F35" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>6202137.05375</v>
+      </c>
+      <c r="G35" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>8369278.62125</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="49" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="B36" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1867853.91875</v>
+      </c>
+      <c r="C36" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3222317.3984375</v>
+      </c>
+      <c r="D36" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>4576780.878125</v>
+      </c>
+      <c r="E36" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>6608476.09765625</v>
+      </c>
+      <c r="F36" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>8640171.3171875</v>
+      </c>
+      <c r="G36" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>11349098.2765625</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="26" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:A25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1536,116 +2890,116 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="33" t="s">
-        <v>48</v>
+      <c r="A1" s="50" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="34"/>
+      <c r="A2" s="51"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="35" t="s">
-        <v>49</v>
+      <c r="A3" s="52" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="34" t="s">
-        <v>50</v>
+      <c r="A4" s="51" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="34"/>
+      <c r="A5" s="51"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="35" t="s">
-        <v>51</v>
+      <c r="A6" s="52" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="34" t="s">
-        <v>52</v>
+      <c r="A7" s="51" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="s">
-        <v>53</v>
+      <c r="A8" s="51" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="34"/>
+      <c r="A9" s="51"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="35" t="s">
-        <v>54</v>
+      <c r="A10" s="52" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34" t="s">
-        <v>55</v>
+      <c r="A11" s="51" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34" t="s">
-        <v>56</v>
+      <c r="A12" s="51" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34" t="s">
-        <v>57</v>
+      <c r="A13" s="51" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34" t="s">
-        <v>58</v>
+      <c r="A14" s="51" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34"/>
+      <c r="A15" s="51"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="35" t="s">
-        <v>59</v>
+      <c r="A16" s="52" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="34" t="s">
-        <v>60</v>
+      <c r="A17" s="51" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="34"/>
+      <c r="A18" s="51"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="35" t="s">
-        <v>61</v>
+      <c r="A19" s="52" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34" t="s">
-        <v>62</v>
+      <c r="A20" s="51" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="34" t="s">
-        <v>63</v>
+      <c r="A21" s="51" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="34" t="s">
-        <v>64</v>
+      <c r="A22" s="51" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="34"/>
+      <c r="A23" s="51"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="35" t="s">
-        <v>65</v>
+      <c r="A24" s="52" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="34" t="s">
-        <v>66</v>
+      <c r="A25" s="51" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Thêm sheet định giá vào mô hình doanh thu
Dựng thang giá từ 299k tới 899k để so lợi nhuận, và bảng riêng đo tác
động của khác biệt sản phẩm lên hai bước phễu ③ và ④.

Kết quả: đỉnh lợi nhuận vẫn ở 399k, vùng 299k-499k chênh nhau dưới
8% nên không cần cân nhắc nhiều. Trong khi đó nếu khác biệt sản phẩm
có tác dụng thật, lợi nhuận tăng 82-212% mà không cần đụng tới giá.

Ghi lại lập luận vì sao khác biệt chưa nên quy thành giá cao hơn lúc
ra mắt, và cách dùng khác biệt để đổi hệ quy chiếu của người mua sang
chi phí thuê gia sư thay vì nâng giá.
</commit_message>
<xml_diff>
--- a/docs/_internal/uoc-tinh-doanh-thu.xlsx
+++ b/docs/_internal/uoc-tinh-doanh-thu.xlsx
@@ -9,9 +9,10 @@
   </bookViews>
   <sheets>
     <sheet name="Mô hình" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Đòn bẩy" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Thuê bao" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Ghi chú" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Định giá" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Đòn bẩy" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Thuê bao" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Ghi chú" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="174">
   <si>
     <t xml:space="preserve">Ước tính doanh thu hàng tháng — Gói Nền tảng 399.000đ</t>
   </si>
@@ -167,6 +168,102 @@
   </si>
   <si>
     <t xml:space="preserve">Ô vàng chữ xanh = bạn sửa. Ô xám/xanh lá = công thức tự tính, đừng gõ đè.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Định giá và doanh thu sau khi tính tới khác biệt sản phẩm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kết luận ngắn: khác biệt của bạn KHÔNG nằm ở chỗ bán được giá cao hơn, mà ở chỗ nhiều người đi tới được chỗ trả tiền hơn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A. THANG GIÁ — giá nào cho lợi nhuận cao nhất?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giá bán một gói</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tỷ lệ chạm paywall → mua ở mức giá này</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ĐÂY LÀ CHỖ YẾU NHẤT CỦA CẢ BẢNG — bạn đang đoán. Chỉ đo được sau khi bán thật.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số đơn / tháng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CÒN LẠI / THÁNG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chênh so với mức cao nhất</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→ Giá cho lợi nhuận cao nhất:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B. NẾU KHÁC BIỆT SẢN PHẨM THẬT SỰ CÓ TÁC DỤNG (giá giữ nguyên 399k)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khác biệt không ăn thua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Có tác dụng vừa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Có tác dụng mạnh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">③ Tỷ lệ đăng ký → học hết Chương 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người học kiểm soát nhịp độ nên ít bỏ giữa chừng hơn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chương 1 miễn phí chính là màn chứng minh khác biệt trước khi trả tiền.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chênh so với cột trái</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đọc hai bảng này cùng nhau</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Bảng A: chênh lệch giữa giá tốt nhất và giá tệ nhất chỉ vài chục phần trăm, và vùng 299k-499k gần như bằng nhau. Nghĩa là chọn sai giá trong khoảng đó KHÔNG phải thảm họa — đừng mất nhiều thời gian cân nhắc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Bảng B: nếu khác biệt sản phẩm có tác dụng thật, lợi nhuận nhân lên nhiều lần. Đây mới là chỗ đáng đổ công.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vì sao khác biệt KHÔNG nên quy thành giá cao hơn — ít nhất là lúc ra mắt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Người mua chưa kiểm chứng được. 'Giải thích nguyên nhân' và 'học theo nhịp của mình' là thứ chỉ cảm nhận được sau khi học, không nhìn thấy trên trang bán hàng. Khóa nào cũng tự nhận như vậy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Chưa có bằng chứng xã hội. Không đánh giá, không ảnh chụp học viên, không video. Giá cao mà không có gì chống lưng thì chỉ làm người ta chần chừ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Vẫn thiếu video quay tay và chấm điểm tự động. Định giá ngang app quốc tế lúc này là bán quá giá trị đang có.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Khác biệt của bạn phát huy tác dụng ở bước ③ và ④, không phải ở mức giá. Chương 1 miễn phí là màn trình diễn khác biệt; nó làm NHIỀU NGƯỜI MUA HƠN chứ không làm mỗi người trả nhiều hơn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khi nào được tăng giá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Khi Giai đoạn 2 hoàn thiện → 599k, thông báo trước, người đã mua giữ nguyên quyền.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Khi có 20-30 đánh giá thật của người học đã đi hết Giai đoạn 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Khi Web MIDI chạy được → lúc đó mới có thứ kiểm chứng được, và mới được định giá ngang tầm app quốc tế.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cách dùng khác biệt cho đúng: đổi hệ quy chiếu, không đổi giá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người mua đang so 399k với các khóa online rẻ tiền. Khác biệt thật của bạn (lộ trình rõ, giải thích nguyên nhân, tự kiểm soát nhịp độ) là những thứ trước nay chỉ CÓ GIÁO VIÊN mới cho được — mà gia sư thì 500k-5tr MỖI THÁNG kèm ràng buộc lịch. Đặt cạnh mốc đó, 399k trả một lần trông rất nhỏ. Đây là cách khác biệt giúp bán được hàng mà không cần nâng giá — và không cần nhắc tên bất kỳ app nào.</t>
   </si>
   <si>
     <t xml:space="preserve">So sánh đòn bẩy — thay đổi nào làm lợi nhuận tăng nhiều nhất?</t>
@@ -455,16 +552,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="#,##0&quot; đ&quot;"/>
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
     <numFmt numFmtId="169" formatCode="0%"/>
-    <numFmt numFmtId="170" formatCode="\+0%;\-0%;0%"/>
+    <numFmt numFmtId="170" formatCode="\+0%;\-0%"/>
+    <numFmt numFmtId="171" formatCode="\+0%;\-0%;0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -568,6 +666,12 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="9"/>
+      <name val="Cambria"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Cambria"/>
       <family val="0"/>
@@ -655,7 +759,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="72">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -788,6 +892,82 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -808,11 +988,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -828,7 +1008,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -836,7 +1016,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1831,6 +2011,404 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:I39"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="33" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="34" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="35" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" s="36" t="n">
+        <v>299000</v>
+      </c>
+      <c r="C5" s="36" t="n">
+        <v>399000</v>
+      </c>
+      <c r="D5" s="36" t="n">
+        <v>499000</v>
+      </c>
+      <c r="E5" s="36" t="n">
+        <v>599000</v>
+      </c>
+      <c r="F5" s="36" t="n">
+        <v>699000</v>
+      </c>
+      <c r="G5" s="36" t="n">
+        <v>899000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" s="38" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C6" s="38" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D6" s="38" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E6" s="38" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F6" s="38" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G6" s="38" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I6" s="39" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="40" t="n">
+        <f aca="false">'Mô hình'!$C$9*B6</f>
+        <v>14.7</v>
+      </c>
+      <c r="C7" s="40" t="n">
+        <f aca="false">'Mô hình'!$C$9*C6</f>
+        <v>11.55</v>
+      </c>
+      <c r="D7" s="40" t="n">
+        <f aca="false">'Mô hình'!$C$9*D6</f>
+        <v>8.925</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <f aca="false">'Mô hình'!$C$9*E6</f>
+        <v>6.825</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <f aca="false">'Mô hình'!$C$9*F6</f>
+        <v>5.25</v>
+      </c>
+      <c r="G7" s="40" t="n">
+        <f aca="false">'Mô hình'!$C$9*G6</f>
+        <v>3.15</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="41" t="n">
+        <f aca="false">B7*B5*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4071146.625</v>
+      </c>
+      <c r="C8" s="41" t="n">
+        <f aca="false">C7*C5*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4268576.8125</v>
+      </c>
+      <c r="D8" s="41" t="n">
+        <f aca="false">D7*D5*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4125123.84375</v>
+      </c>
+      <c r="E8" s="41" t="n">
+        <f aca="false">E7*E5*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>3786672.09375</v>
+      </c>
+      <c r="F8" s="41" t="n">
+        <f aca="false">F7*F5*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>3399105.9375</v>
+      </c>
+      <c r="G8" s="41" t="n">
+        <f aca="false">G7*G5*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>2623001.0625</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="42" t="n">
+        <f aca="false">B8-'Mô hình'!$C$25-B8*'Mô hình'!$C$26</f>
+        <v>2236166.36125</v>
+      </c>
+      <c r="C9" s="42" t="n">
+        <f aca="false">C8-'Mô hình'!$C$25-C8*'Mô hình'!$C$26</f>
+        <v>2419776.435625</v>
+      </c>
+      <c r="D9" s="42" t="n">
+        <f aca="false">D8-'Mô hình'!$C$25-D8*'Mô hình'!$C$26</f>
+        <v>2286365.1746875</v>
+      </c>
+      <c r="E9" s="42" t="n">
+        <f aca="false">E8-'Mô hình'!$C$25-E8*'Mô hình'!$C$26</f>
+        <v>1971605.0471875</v>
+      </c>
+      <c r="F9" s="42" t="n">
+        <f aca="false">F8-'Mô hình'!$C$25-F8*'Mô hình'!$C$26</f>
+        <v>1611168.521875</v>
+      </c>
+      <c r="G9" s="42" t="n">
+        <f aca="false">G8-'Mô hình'!$C$25-G8*'Mô hình'!$C$26</f>
+        <v>889390.988125</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="43" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="44" t="n">
+        <f aca="false">B9/MAX($B$9:$G$9)-1</f>
+        <v>-0.0758789414062444</v>
+      </c>
+      <c r="C10" s="44" t="n">
+        <f aca="false">C9/MAX($B$9:$G$9)-1</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="44" t="n">
+        <f aca="false">D9/MAX($B$9:$G$9)-1</f>
+        <v>-0.055133713583355</v>
+      </c>
+      <c r="E10" s="44" t="n">
+        <f aca="false">E9/MAX($B$9:$G$9)-1</f>
+        <v>-0.185211898851202</v>
+      </c>
+      <c r="F10" s="44" t="n">
+        <f aca="false">F9/MAX($B$9:$G$9)-1</f>
+        <v>-0.334166372498436</v>
+      </c>
+      <c r="G10" s="44" t="n">
+        <f aca="false">G9/MAX($B$9:$G$9)-1</f>
+        <v>-0.632449107681603</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="42" t="n">
+        <f aca="false">INDEX($B$5:$G$5,MATCH(MAX($B$9:$G$9),$B$9:$G$9,0))</f>
+        <v>399000</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="35" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="45"/>
+      <c r="B15" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="46" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16" s="38" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C16" s="38" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D16" s="38" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F16" s="47" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="38" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="C17" s="38" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D17" s="38" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F17" s="47" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="49" t="n">
+        <f aca="false">'Mô hình'!$C$7*B16*B17</f>
+        <v>11.55</v>
+      </c>
+      <c r="C18" s="49" t="n">
+        <f aca="false">'Mô hình'!$C$7*C16*C17</f>
+        <v>17.325</v>
+      </c>
+      <c r="D18" s="49" t="n">
+        <f aca="false">'Mô hình'!$C$7*D16*D17</f>
+        <v>26.46</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="50" t="n">
+        <f aca="false">B18*399000*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4268576.8125</v>
+      </c>
+      <c r="C19" s="50" t="n">
+        <f aca="false">C18*399000*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>6402865.21875</v>
+      </c>
+      <c r="D19" s="50" t="n">
+        <f aca="false">D18*399000*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>9778921.425</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="42" t="n">
+        <f aca="false">B19-'Mô hình'!$C$25-B19*'Mô hình'!$C$26</f>
+        <v>2419776.435625</v>
+      </c>
+      <c r="C20" s="42" t="n">
+        <f aca="false">C19-'Mô hình'!$C$25-C19*'Mô hình'!$C$26</f>
+        <v>4404664.6534375</v>
+      </c>
+      <c r="D20" s="42" t="n">
+        <f aca="false">D19-'Mô hình'!$C$25-D19*'Mô hình'!$C$26</f>
+        <v>7544396.92525</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="43" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="51"/>
+      <c r="C21" s="51" t="n">
+        <f aca="false">C20/$B$20-1</f>
+        <v>0.820277521753709</v>
+      </c>
+      <c r="D21" s="51" t="n">
+        <f aca="false">D20/$B$20-1</f>
+        <v>2.11780741980049</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="35" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="35" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="35" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:L21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1849,66 +2427,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>48</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="32" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="33" t="s">
-        <v>50</v>
-      </c>
-      <c r="B4" s="33" t="s">
-        <v>51</v>
-      </c>
-      <c r="C4" s="33" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="E4" s="33" t="s">
-        <v>54</v>
-      </c>
-      <c r="F4" s="33" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" s="33" t="s">
-        <v>56</v>
-      </c>
-      <c r="H4" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="I4" s="33" t="s">
-        <v>58</v>
-      </c>
-      <c r="J4" s="33" t="s">
-        <v>59</v>
-      </c>
-      <c r="K4" s="33" t="s">
-        <v>60</v>
-      </c>
-      <c r="L4" s="33" t="s">
-        <v>61</v>
+      <c r="A4" s="52" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="52" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="52" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="52" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="52" t="s">
+        <v>86</v>
+      </c>
+      <c r="F4" s="52" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="52" t="s">
+        <v>88</v>
+      </c>
+      <c r="H4" s="52" t="s">
+        <v>89</v>
+      </c>
+      <c r="I4" s="52" t="s">
+        <v>90</v>
+      </c>
+      <c r="J4" s="52" t="s">
+        <v>91</v>
+      </c>
+      <c r="K4" s="52" t="s">
+        <v>92</v>
+      </c>
+      <c r="L4" s="52" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="34" t="s">
-        <v>62</v>
+      <c r="A5" s="53" t="s">
+        <v>94</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>3000</v>
       </c>
-      <c r="C5" s="35" t="n">
+      <c r="C5" s="54" t="n">
         <v>0.07</v>
       </c>
-      <c r="D5" s="35" t="n">
+      <c r="D5" s="54" t="n">
         <v>0.25</v>
       </c>
-      <c r="E5" s="35" t="n">
+      <c r="E5" s="54" t="n">
         <v>0.22</v>
       </c>
       <c r="F5" s="21" t="n">
@@ -1920,11 +2498,11 @@
       <c r="H5" s="21" t="n">
         <v>1550000</v>
       </c>
-      <c r="I5" s="36" t="n">
+      <c r="I5" s="55" t="n">
         <f aca="false">B5*C5*D5*E5</f>
         <v>11.55</v>
       </c>
-      <c r="J5" s="37" t="n">
+      <c r="J5" s="56" t="n">
         <f aca="false">I5*(F5+G5)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
         <v>4268576.8125</v>
       </c>
@@ -1932,25 +2510,25 @@
         <f aca="false">J5-H5-J5*'Mô hình'!$C$26</f>
         <v>2419776.435625</v>
       </c>
-      <c r="L5" s="38" t="n">
+      <c r="L5" s="57" t="n">
         <f aca="false">IF($K$5=0,"",K5/$K$5-1)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="39" t="s">
-        <v>63</v>
+      <c r="A6" s="58" t="s">
+        <v>95</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>3000</v>
       </c>
-      <c r="C6" s="40" t="n">
+      <c r="C6" s="59" t="n">
         <v>0.07</v>
       </c>
-      <c r="D6" s="40" t="n">
+      <c r="D6" s="59" t="n">
         <v>0.25</v>
       </c>
-      <c r="E6" s="40" t="n">
+      <c r="E6" s="59" t="n">
         <v>0.22</v>
       </c>
       <c r="F6" s="15" t="n">
@@ -1962,11 +2540,11 @@
       <c r="H6" s="15" t="n">
         <v>1550000</v>
       </c>
-      <c r="I6" s="41" t="n">
+      <c r="I6" s="60" t="n">
         <f aca="false">B6*C6*D6*E6</f>
         <v>11.55</v>
       </c>
-      <c r="J6" s="42" t="n">
+      <c r="J6" s="61" t="n">
         <f aca="false">I6*(F6+G6)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
         <v>6408214.3125</v>
       </c>
@@ -1974,25 +2552,25 @@
         <f aca="false">J6-H6-J6*'Mô hình'!$C$26</f>
         <v>4409639.310625</v>
       </c>
-      <c r="L6" s="43" t="n">
+      <c r="L6" s="62" t="n">
         <f aca="false">IF($K$5=0,"",K6/$K$5-1)</f>
         <v>0.822333355141564</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="39" t="s">
-        <v>64</v>
+      <c r="A7" s="58" t="s">
+        <v>96</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>3000</v>
       </c>
-      <c r="C7" s="40" t="n">
+      <c r="C7" s="59" t="n">
         <v>0.07</v>
       </c>
-      <c r="D7" s="40" t="n">
+      <c r="D7" s="59" t="n">
         <v>0.25</v>
       </c>
-      <c r="E7" s="40" t="n">
+      <c r="E7" s="59" t="n">
         <v>0.165</v>
       </c>
       <c r="F7" s="15" t="n">
@@ -2004,11 +2582,11 @@
       <c r="H7" s="15" t="n">
         <v>1550000</v>
       </c>
-      <c r="I7" s="41" t="n">
+      <c r="I7" s="60" t="n">
         <f aca="false">B7*C7*D7*E7</f>
         <v>8.6625</v>
       </c>
-      <c r="J7" s="42" t="n">
+      <c r="J7" s="61" t="n">
         <f aca="false">I7*(F7+G7)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
         <v>4806160.734375</v>
       </c>
@@ -2016,25 +2594,25 @@
         <f aca="false">J7-H7-J7*'Mô hình'!$C$26</f>
         <v>2919729.48296875</v>
       </c>
-      <c r="L7" s="43" t="n">
+      <c r="L7" s="62" t="n">
         <f aca="false">IF($K$5=0,"",K7/$K$5-1)</f>
         <v>0.206611255479318</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="39" t="s">
-        <v>65</v>
+      <c r="A8" s="58" t="s">
+        <v>97</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>3000</v>
       </c>
-      <c r="C8" s="40" t="n">
+      <c r="C8" s="59" t="n">
         <v>0.07</v>
       </c>
-      <c r="D8" s="40" t="n">
+      <c r="D8" s="59" t="n">
         <v>0.4</v>
       </c>
-      <c r="E8" s="40" t="n">
+      <c r="E8" s="59" t="n">
         <v>0.22</v>
       </c>
       <c r="F8" s="15" t="n">
@@ -2046,11 +2624,11 @@
       <c r="H8" s="15" t="n">
         <v>1550000</v>
       </c>
-      <c r="I8" s="41" t="n">
+      <c r="I8" s="60" t="n">
         <f aca="false">B8*C8*D8*E8</f>
         <v>18.48</v>
       </c>
-      <c r="J8" s="42" t="n">
+      <c r="J8" s="61" t="n">
         <f aca="false">I8*(F8+G8)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
         <v>6829722.9</v>
       </c>
@@ -2058,25 +2636,25 @@
         <f aca="false">J8-H8-J8*'Mô hình'!$C$26</f>
         <v>4801642.297</v>
       </c>
-      <c r="L8" s="43" t="n">
+      <c r="L8" s="62" t="n">
         <f aca="false">IF($K$5=0,"",K8/$K$5-1)</f>
         <v>0.984333026104451</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="39" t="s">
-        <v>66</v>
+      <c r="A9" s="58" t="s">
+        <v>98</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>3000</v>
       </c>
-      <c r="C9" s="40" t="n">
+      <c r="C9" s="59" t="n">
         <v>0.07</v>
       </c>
-      <c r="D9" s="40" t="n">
+      <c r="D9" s="59" t="n">
         <v>0.25</v>
       </c>
-      <c r="E9" s="40" t="n">
+      <c r="E9" s="59" t="n">
         <v>0.22</v>
       </c>
       <c r="F9" s="15" t="n">
@@ -2088,11 +2666,11 @@
       <c r="H9" s="15" t="n">
         <v>1550000</v>
       </c>
-      <c r="I9" s="41" t="n">
+      <c r="I9" s="60" t="n">
         <f aca="false">B9*C9*D9*E9</f>
         <v>11.55</v>
       </c>
-      <c r="J9" s="42" t="n">
+      <c r="J9" s="61" t="n">
         <f aca="false">I9*(F9+G9)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
         <v>6194250.5625</v>
       </c>
@@ -2100,25 +2678,25 @@
         <f aca="false">J9-H9-J9*'Mô hình'!$C$26</f>
         <v>4210653.023125</v>
       </c>
-      <c r="L9" s="43" t="n">
+      <c r="L9" s="62" t="n">
         <f aca="false">IF($K$5=0,"",K9/$K$5-1)</f>
         <v>0.740100019627408</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="39" t="s">
-        <v>67</v>
+      <c r="A10" s="58" t="s">
+        <v>99</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>3000</v>
       </c>
-      <c r="C10" s="40" t="n">
+      <c r="C10" s="59" t="n">
         <v>0.07</v>
       </c>
-      <c r="D10" s="40" t="n">
+      <c r="D10" s="59" t="n">
         <v>0.25</v>
       </c>
-      <c r="E10" s="40" t="n">
+      <c r="E10" s="59" t="n">
         <v>0.22</v>
       </c>
       <c r="F10" s="15" t="n">
@@ -2130,11 +2708,11 @@
       <c r="H10" s="15" t="n">
         <v>1750000</v>
       </c>
-      <c r="I10" s="41" t="n">
+      <c r="I10" s="60" t="n">
         <f aca="false">B10*C10*D10*E10</f>
         <v>11.55</v>
       </c>
-      <c r="J10" s="42" t="n">
+      <c r="J10" s="61" t="n">
         <f aca="false">I10*(F10+G10)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
         <v>5338395.5625</v>
       </c>
@@ -2142,25 +2720,25 @@
         <f aca="false">J10-H10-J10*'Mô hình'!$C$26</f>
         <v>3214707.873125</v>
       </c>
-      <c r="L10" s="43" t="n">
+      <c r="L10" s="62" t="n">
         <f aca="false">IF($K$5=0,"",K10/$K$5-1)</f>
         <v>0.328514413892405</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="39" t="s">
-        <v>68</v>
+      <c r="A11" s="58" t="s">
+        <v>100</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>2100</v>
       </c>
-      <c r="C11" s="40" t="n">
+      <c r="C11" s="59" t="n">
         <v>0.07</v>
       </c>
-      <c r="D11" s="40" t="n">
+      <c r="D11" s="59" t="n">
         <v>0.25</v>
       </c>
-      <c r="E11" s="40" t="n">
+      <c r="E11" s="59" t="n">
         <v>0.22</v>
       </c>
       <c r="F11" s="15" t="n">
@@ -2172,11 +2750,11 @@
       <c r="H11" s="15" t="n">
         <v>550000</v>
       </c>
-      <c r="I11" s="41" t="n">
+      <c r="I11" s="60" t="n">
         <f aca="false">B11*C11*D11*E11</f>
         <v>8.085</v>
       </c>
-      <c r="J11" s="42" t="n">
+      <c r="J11" s="61" t="n">
         <f aca="false">I11*(F11+G11)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
         <v>2988003.76875</v>
       </c>
@@ -2184,25 +2762,25 @@
         <f aca="false">J11-H11-J11*'Mô hình'!$C$26</f>
         <v>2228843.5049375</v>
       </c>
-      <c r="L11" s="43" t="n">
+      <c r="L11" s="62" t="n">
         <f aca="false">IF($K$5=0,"",K11/$K$5-1)</f>
         <v>-0.0789051946603426</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="39" t="s">
-        <v>69</v>
+      <c r="A12" s="58" t="s">
+        <v>101</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>6000</v>
       </c>
-      <c r="C12" s="40" t="n">
+      <c r="C12" s="59" t="n">
         <v>0.07</v>
       </c>
-      <c r="D12" s="40" t="n">
+      <c r="D12" s="59" t="n">
         <v>0.25</v>
       </c>
-      <c r="E12" s="40" t="n">
+      <c r="E12" s="59" t="n">
         <v>0.22</v>
       </c>
       <c r="F12" s="15" t="n">
@@ -2214,11 +2792,11 @@
       <c r="H12" s="15" t="n">
         <v>3550000</v>
       </c>
-      <c r="I12" s="41" t="n">
+      <c r="I12" s="60" t="n">
         <f aca="false">B12*C12*D12*E12</f>
         <v>23.1</v>
       </c>
-      <c r="J12" s="42" t="n">
+      <c r="J12" s="61" t="n">
         <f aca="false">I12*(F12+G12)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
         <v>8537153.625</v>
       </c>
@@ -2226,25 +2804,25 @@
         <f aca="false">J12-H12-J12*'Mô hình'!$C$26</f>
         <v>4389552.87125</v>
       </c>
-      <c r="L12" s="43" t="n">
+      <c r="L12" s="62" t="n">
         <f aca="false">IF($K$5=0,"",K12/$K$5-1)</f>
         <v>0.814032406723652</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="39" t="s">
-        <v>70</v>
+      <c r="A13" s="58" t="s">
+        <v>102</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>3000</v>
       </c>
-      <c r="C13" s="40" t="n">
+      <c r="C13" s="59" t="n">
         <v>0.07</v>
       </c>
-      <c r="D13" s="40" t="n">
+      <c r="D13" s="59" t="n">
         <v>0.4</v>
       </c>
-      <c r="E13" s="40" t="n">
+      <c r="E13" s="59" t="n">
         <v>0.22</v>
       </c>
       <c r="F13" s="15" t="n">
@@ -2256,11 +2834,11 @@
       <c r="H13" s="15" t="n">
         <v>1550000</v>
       </c>
-      <c r="I13" s="41" t="n">
+      <c r="I13" s="60" t="n">
         <f aca="false">B13*C13*D13*E13</f>
         <v>18.48</v>
       </c>
-      <c r="J13" s="42" t="n">
+      <c r="J13" s="61" t="n">
         <f aca="false">I13*(F13+G13)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
         <v>14874759.9</v>
       </c>
@@ -2268,603 +2846,39 @@
         <f aca="false">J13-H13-J13*'Mô hình'!$C$26</f>
         <v>12283526.707</v>
       </c>
-      <c r="L13" s="43" t="n">
+      <c r="L13" s="62" t="n">
         <f aca="false">IF($K$5=0,"",K13/$K$5-1)</f>
         <v>4.07630644143673</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="26" t="s">
-        <v>71</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>72</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>73</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>74</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>75</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:G42"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="1" width="16"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="32" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" s="18"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="44" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="8" t="n">
-        <f aca="false">'Mô hình'!C9</f>
-        <v>52.5</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="44" t="s">
-        <v>83</v>
-      </c>
-      <c r="B6" s="40" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="44" t="s">
-        <v>85</v>
-      </c>
-      <c r="B7" s="40" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="B8" s="15" t="n">
-        <v>399000</v>
-      </c>
-      <c r="D8" s="9"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="44" t="s">
-        <v>88</v>
-      </c>
-      <c r="B9" s="15" t="n">
-        <v>599000</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="44" t="s">
-        <v>90</v>
-      </c>
-      <c r="B10" s="40" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="44" t="s">
-        <v>92</v>
-      </c>
-      <c r="B11" s="15" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="44" t="s">
-        <v>94</v>
-      </c>
-      <c r="B12" s="15" t="n">
-        <v>1550000</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="45" t="s">
-        <v>99</v>
-      </c>
-      <c r="B15" s="36" t="n">
-        <f aca="false">$B$5*$B$6</f>
-        <v>11.55</v>
-      </c>
-      <c r="C15" s="36" t="n">
-        <f aca="false">$B$5*$B$7</f>
-        <v>7.875</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="45" t="s">
-        <v>100</v>
-      </c>
-      <c r="B16" s="37" t="n">
-        <f aca="false">B15*$B$8*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
-        <v>4268576.8125</v>
-      </c>
-      <c r="C16" s="37" t="n">
-        <f aca="false">C15*$B$9*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
-        <v>4369237.03125</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="26" t="s">
-        <v>102</v>
-      </c>
-      <c r="B17" s="20" t="n">
-        <f aca="false">B15*$B$8*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
-        <v>4268576.8125</v>
-      </c>
-      <c r="C17" s="20" t="n">
-        <f aca="false">C15*$B$9/(1-$B$10)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
-        <v>6721903.125</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="B18" s="46" t="s">
-        <v>105</v>
-      </c>
-      <c r="C18" s="47" t="n">
-        <f aca="false">C15*12/(1-$B$10)</f>
-        <v>145.384615384615</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="45" t="s">
-        <v>107</v>
-      </c>
-      <c r="B19" s="37" t="n">
-        <f aca="false">$B$8</f>
-        <v>399000</v>
-      </c>
-      <c r="C19" s="37" t="n">
-        <f aca="false">$B$9/(1-$B$10)</f>
-        <v>921538.461538462</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="45" t="s">
         <v>108</v>
-      </c>
-      <c r="B20" s="37" t="n">
-        <f aca="false">$B$12</f>
-        <v>1550000</v>
-      </c>
-      <c r="C20" s="37" t="n">
-        <f aca="false">$B$11+$B$12</f>
-        <v>3550000</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="B21" s="20" t="n">
-        <f aca="false">B16-B20-B16*'Mô hình'!$C$26</f>
-        <v>2419776.435625</v>
-      </c>
-      <c r="C21" s="20" t="n">
-        <f aca="false">C16-C20-C16*'Mô hình'!$C$26</f>
-        <v>513390.439062501</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="26" t="s">
-        <v>111</v>
-      </c>
-      <c r="B22" s="20" t="n">
-        <f aca="false">B17-B20-B17*'Mô hình'!$C$26</f>
-        <v>2419776.435625</v>
-      </c>
-      <c r="C22" s="20" t="n">
-        <f aca="false">C17-C20-C17*'Mô hình'!$C$26</f>
-        <v>2701369.90625</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="26" t="s">
-        <v>112</v>
-      </c>
-      <c r="B24" s="48" t="n">
-        <f aca="false">IF(C15=0,"",1-(C15*$B$9*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)*(1-'Mô hình'!$C$26))/(B15*$B$8*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)*(1-'Mô hình'!$C$26)+$B$11))</f>
-        <v>0.319339596234463</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="45" t="s">
-        <v>114</v>
-      </c>
-      <c r="B25" s="37" t="n">
-        <f aca="false">$B$11/(1-'Mô hình'!$C$26)</f>
-        <v>2150537.6344086</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="26" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="28" t="s">
-        <v>117</v>
-      </c>
-      <c r="B28" s="29" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="C28" s="29" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D28" s="29" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="E28" s="29" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F28" s="29" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G28" s="29" t="n">
-        <v>0.22</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="49" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="B29" s="31" t="n">
-        <f aca="false">($B$5*B$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>-1000421.68529412</v>
-      </c>
-      <c r="C29" s="31" t="n">
-        <f aca="false">($B$5*C$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>-363027.106617647</v>
-      </c>
-      <c r="D29" s="31" t="n">
-        <f aca="false">($B$5*D$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>274367.472058824</v>
-      </c>
-      <c r="E29" s="31" t="n">
-        <f aca="false">($B$5*E$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>1230459.34007353</v>
-      </c>
-      <c r="F29" s="31" t="n">
-        <f aca="false">($B$5*F$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>2186551.20808824</v>
-      </c>
-      <c r="G29" s="31" t="n">
-        <f aca="false">($B$5*G$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>3461340.36544118</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="49" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="B30" s="31" t="n">
-        <f aca="false">($B$5*B$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>-841073.040625</v>
-      </c>
-      <c r="C30" s="31" t="n">
-        <f aca="false">($B$5*C$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>-163841.30078125</v>
-      </c>
-      <c r="D30" s="31" t="n">
-        <f aca="false">($B$5*D$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>513390.4390625</v>
-      </c>
-      <c r="E30" s="31" t="n">
-        <f aca="false">($B$5*E$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>1529238.04882813</v>
-      </c>
-      <c r="F30" s="31" t="n">
-        <f aca="false">($B$5*F$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>2545085.65859375</v>
-      </c>
-      <c r="G30" s="31" t="n">
-        <f aca="false">($B$5*G$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>3899549.13828125</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="49" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="B31" s="31" t="n">
-        <f aca="false">($B$5*B$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>-660477.91</v>
-      </c>
-      <c r="C31" s="31" t="n">
-        <f aca="false">($B$5*C$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>61902.6125000003</v>
-      </c>
-      <c r="D31" s="31" t="n">
-        <f aca="false">($B$5*D$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>784283.135000001</v>
-      </c>
-      <c r="E31" s="31" t="n">
-        <f aca="false">($B$5*E$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>1867853.91875</v>
-      </c>
-      <c r="F31" s="31" t="n">
-        <f aca="false">($B$5*F$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>2951424.7025</v>
-      </c>
-      <c r="G31" s="31" t="n">
-        <f aca="false">($B$5*G$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>4396185.7475</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="49" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="B32" s="31" t="n">
-        <f aca="false">($B$5*B$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>-454083.474999999</v>
-      </c>
-      <c r="C32" s="31" t="n">
-        <f aca="false">($B$5*C$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>319895.65625</v>
-      </c>
-      <c r="D32" s="31" t="n">
-        <f aca="false">($B$5*D$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>1093874.7875</v>
-      </c>
-      <c r="E32" s="31" t="n">
-        <f aca="false">($B$5*E$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>2254843.484375</v>
-      </c>
-      <c r="F32" s="31" t="n">
-        <f aca="false">($B$5*F$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>3415812.18125</v>
-      </c>
-      <c r="G32" s="31" t="n">
-        <f aca="false">($B$5*G$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>4963770.44375</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="49" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="B33" s="31" t="n">
-        <f aca="false">($B$5*B$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>-215936.05</v>
-      </c>
-      <c r="C33" s="31" t="n">
-        <f aca="false">($B$5*C$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>617579.937500001</v>
-      </c>
-      <c r="D33" s="31" t="n">
-        <f aca="false">($B$5*D$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>1451095.925</v>
-      </c>
-      <c r="E33" s="31" t="n">
-        <f aca="false">($B$5*E$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>2701369.90625</v>
-      </c>
-      <c r="F33" s="31" t="n">
-        <f aca="false">($B$5*F$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>3951643.8875</v>
-      </c>
-      <c r="G33" s="31" t="n">
-        <f aca="false">($B$5*G$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>5618675.8625</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="49" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="B34" s="31" t="n">
-        <f aca="false">($B$5*B$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>61902.6125000007</v>
-      </c>
-      <c r="C34" s="31" t="n">
-        <f aca="false">($B$5*C$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>964878.265625001</v>
-      </c>
-      <c r="D34" s="31" t="n">
-        <f aca="false">($B$5*D$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>1867853.91875</v>
-      </c>
-      <c r="E34" s="31" t="n">
-        <f aca="false">($B$5*E$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>3222317.3984375</v>
-      </c>
-      <c r="F34" s="31" t="n">
-        <f aca="false">($B$5*F$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>4576780.878125</v>
-      </c>
-      <c r="G34" s="31" t="n">
-        <f aca="false">($B$5*G$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>6382732.184375</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="49" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B35" s="31" t="n">
-        <f aca="false">($B$5*B$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>784283.135000001</v>
-      </c>
-      <c r="C35" s="31" t="n">
-        <f aca="false">($B$5*C$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>1867853.91875</v>
-      </c>
-      <c r="D35" s="31" t="n">
-        <f aca="false">($B$5*D$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>2951424.7025</v>
-      </c>
-      <c r="E35" s="31" t="n">
-        <f aca="false">($B$5*E$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>4576780.878125</v>
-      </c>
-      <c r="F35" s="31" t="n">
-        <f aca="false">($B$5*F$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>6202137.05375</v>
-      </c>
-      <c r="G35" s="31" t="n">
-        <f aca="false">($B$5*G$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>8369278.62125</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="49" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="B36" s="31" t="n">
-        <f aca="false">($B$5*B$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>1867853.91875</v>
-      </c>
-      <c r="C36" s="31" t="n">
-        <f aca="false">($B$5*C$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>3222317.3984375</v>
-      </c>
-      <c r="D36" s="31" t="n">
-        <f aca="false">($B$5*D$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>4576780.878125</v>
-      </c>
-      <c r="E36" s="31" t="n">
-        <f aca="false">($B$5*E$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>6608476.09765625</v>
-      </c>
-      <c r="F36" s="31" t="n">
-        <f aca="false">($B$5*F$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>8640171.3171875</v>
-      </c>
-      <c r="G36" s="31" t="n">
-        <f aca="false">($B$5*G$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
-        <v>11349098.2765625</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="26" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -2883,6 +2897,570 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:G42"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="1" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="32" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="C4" s="18"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="63" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="8" t="n">
+        <f aca="false">'Mô hình'!C9</f>
+        <v>52.5</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="63" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" s="59" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="63" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="59" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="63" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>399000</v>
+      </c>
+      <c r="D8" s="9"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="63" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>599000</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="63" t="s">
+        <v>122</v>
+      </c>
+      <c r="B10" s="59" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="63" t="s">
+        <v>124</v>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="63" t="s">
+        <v>126</v>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>1550000</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="64" t="s">
+        <v>131</v>
+      </c>
+      <c r="B15" s="55" t="n">
+        <f aca="false">$B$5*$B$6</f>
+        <v>11.55</v>
+      </c>
+      <c r="C15" s="55" t="n">
+        <f aca="false">$B$5*$B$7</f>
+        <v>7.875</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="64" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" s="56" t="n">
+        <f aca="false">B15*$B$8*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4268576.8125</v>
+      </c>
+      <c r="C16" s="56" t="n">
+        <f aca="false">C15*$B$9*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4369237.03125</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="26" t="s">
+        <v>134</v>
+      </c>
+      <c r="B17" s="20" t="n">
+        <f aca="false">B15*$B$8*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>4268576.8125</v>
+      </c>
+      <c r="C17" s="20" t="n">
+        <f aca="false">C15*$B$9/(1-$B$10)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)</f>
+        <v>6721903.125</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="64" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" s="65" t="s">
+        <v>137</v>
+      </c>
+      <c r="C18" s="66" t="n">
+        <f aca="false">C15*12/(1-$B$10)</f>
+        <v>145.384615384615</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="64" t="s">
+        <v>139</v>
+      </c>
+      <c r="B19" s="56" t="n">
+        <f aca="false">$B$8</f>
+        <v>399000</v>
+      </c>
+      <c r="C19" s="56" t="n">
+        <f aca="false">$B$9/(1-$B$10)</f>
+        <v>921538.461538462</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="64" t="s">
+        <v>140</v>
+      </c>
+      <c r="B20" s="56" t="n">
+        <f aca="false">$B$12</f>
+        <v>1550000</v>
+      </c>
+      <c r="C20" s="56" t="n">
+        <f aca="false">$B$11+$B$12</f>
+        <v>3550000</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="26" t="s">
+        <v>142</v>
+      </c>
+      <c r="B21" s="20" t="n">
+        <f aca="false">B16-B20-B16*'Mô hình'!$C$26</f>
+        <v>2419776.435625</v>
+      </c>
+      <c r="C21" s="20" t="n">
+        <f aca="false">C16-C20-C16*'Mô hình'!$C$26</f>
+        <v>513390.439062501</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="26" t="s">
+        <v>143</v>
+      </c>
+      <c r="B22" s="20" t="n">
+        <f aca="false">B17-B20-B17*'Mô hình'!$C$26</f>
+        <v>2419776.435625</v>
+      </c>
+      <c r="C22" s="20" t="n">
+        <f aca="false">C17-C20-C17*'Mô hình'!$C$26</f>
+        <v>2701369.90625</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="B24" s="67" t="n">
+        <f aca="false">IF(C15=0,"",1-(C15*$B$9*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)*(1-'Mô hình'!$C$26))/(B15*$B$8*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17)*(1-'Mô hình'!$C$26)+$B$11))</f>
+        <v>0.319339596234463</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="64" t="s">
+        <v>146</v>
+      </c>
+      <c r="B25" s="56" t="n">
+        <f aca="false">$B$11/(1-'Mô hình'!$C$26)</f>
+        <v>2150537.6344086</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="26" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="28" t="s">
+        <v>149</v>
+      </c>
+      <c r="B28" s="29" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C28" s="29" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D28" s="29" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E28" s="29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F28" s="29" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G28" s="29" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="68" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="B29" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-1000421.68529412</v>
+      </c>
+      <c r="C29" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-363027.106617647</v>
+      </c>
+      <c r="D29" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>274367.472058824</v>
+      </c>
+      <c r="E29" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1230459.34007353</v>
+      </c>
+      <c r="F29" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2186551.20808824</v>
+      </c>
+      <c r="G29" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A29)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3461340.36544118</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="68" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B30" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-841073.040625</v>
+      </c>
+      <c r="C30" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-163841.30078125</v>
+      </c>
+      <c r="D30" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>513390.4390625</v>
+      </c>
+      <c r="E30" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1529238.04882813</v>
+      </c>
+      <c r="F30" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2545085.65859375</v>
+      </c>
+      <c r="G30" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A30)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3899549.13828125</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="68" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B31" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-660477.91</v>
+      </c>
+      <c r="C31" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>61902.6125000003</v>
+      </c>
+      <c r="D31" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>784283.135000001</v>
+      </c>
+      <c r="E31" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1867853.91875</v>
+      </c>
+      <c r="F31" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2951424.7025</v>
+      </c>
+      <c r="G31" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A31)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>4396185.7475</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="68" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B32" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-454083.474999999</v>
+      </c>
+      <c r="C32" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>319895.65625</v>
+      </c>
+      <c r="D32" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1093874.7875</v>
+      </c>
+      <c r="E32" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2254843.484375</v>
+      </c>
+      <c r="F32" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3415812.18125</v>
+      </c>
+      <c r="G32" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A32)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>4963770.44375</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="68" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B33" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>-215936.05</v>
+      </c>
+      <c r="C33" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>617579.937500001</v>
+      </c>
+      <c r="D33" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1451095.925</v>
+      </c>
+      <c r="E33" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2701369.90625</v>
+      </c>
+      <c r="F33" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3951643.8875</v>
+      </c>
+      <c r="G33" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A33)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>5618675.8625</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="68" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B34" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>61902.6125000007</v>
+      </c>
+      <c r="C34" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>964878.265625001</v>
+      </c>
+      <c r="D34" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1867853.91875</v>
+      </c>
+      <c r="E34" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3222317.3984375</v>
+      </c>
+      <c r="F34" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>4576780.878125</v>
+      </c>
+      <c r="G34" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A34)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>6382732.184375</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="68" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B35" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>784283.135000001</v>
+      </c>
+      <c r="C35" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1867853.91875</v>
+      </c>
+      <c r="D35" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>2951424.7025</v>
+      </c>
+      <c r="E35" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>4576780.878125</v>
+      </c>
+      <c r="F35" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>6202137.05375</v>
+      </c>
+      <c r="G35" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A35)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>8369278.62125</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="68" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="B36" s="31" t="n">
+        <f aca="false">($B$5*B$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>1867853.91875</v>
+      </c>
+      <c r="C36" s="31" t="n">
+        <f aca="false">($B$5*C$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>3222317.3984375</v>
+      </c>
+      <c r="D36" s="31" t="n">
+        <f aca="false">($B$5*D$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>4576780.878125</v>
+      </c>
+      <c r="E36" s="31" t="n">
+        <f aca="false">($B$5*E$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>6608476.09765625</v>
+      </c>
+      <c r="F36" s="31" t="n">
+        <f aca="false">($B$5*F$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>8640171.3171875</v>
+      </c>
+      <c r="G36" s="31" t="n">
+        <f aca="false">($B$5*G$28*$B$9/(1-$A36)*(1-'Mô hình'!$C$16)*(1-'Mô hình'!$C$17))*(1-'Mô hình'!$C$26)-($B$11+$B$12)</f>
+        <v>11349098.2765625</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="26" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:A25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2890,116 +3468,116 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="50" t="s">
-        <v>123</v>
+      <c r="A1" s="69" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="51"/>
+      <c r="A2" s="70"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="52" t="s">
-        <v>124</v>
+      <c r="A3" s="71" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="51" t="s">
-        <v>125</v>
+      <c r="A4" s="70" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="51"/>
+      <c r="A5" s="70"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="52" t="s">
-        <v>126</v>
+      <c r="A6" s="71" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="51" t="s">
-        <v>127</v>
+      <c r="A7" s="70" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="51" t="s">
-        <v>128</v>
+      <c r="A8" s="70" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="51"/>
+      <c r="A9" s="70"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="52" t="s">
-        <v>129</v>
+      <c r="A10" s="71" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="51" t="s">
-        <v>130</v>
+      <c r="A11" s="70" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="51" t="s">
-        <v>131</v>
+      <c r="A12" s="70" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="51" t="s">
-        <v>132</v>
+      <c r="A13" s="70" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="51" t="s">
-        <v>133</v>
+      <c r="A14" s="70" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="51"/>
+      <c r="A15" s="70"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="52" t="s">
-        <v>134</v>
+      <c r="A16" s="71" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="51" t="s">
-        <v>135</v>
+      <c r="A17" s="70" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="51"/>
+      <c r="A18" s="70"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="52" t="s">
-        <v>136</v>
+      <c r="A19" s="71" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="51" t="s">
-        <v>137</v>
+      <c r="A20" s="70" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="51" t="s">
-        <v>138</v>
+      <c r="A21" s="70" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="51" t="s">
-        <v>139</v>
+      <c r="A22" s="70" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="51"/>
+      <c r="A23" s="70"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="52" t="s">
-        <v>140</v>
+      <c r="A24" s="71" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="51" t="s">
-        <v>141</v>
+      <c r="A25" s="70" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>